<commit_message>
v26.09.7: 升级 MXU v2.5.3 + MaaFramework v5.13.0
* 底层：MXU v1.13.1 -> v2.5.3；MaaFramework v5.7.0-alpha.2 -> v5.13.0
* 移除过期兜底（Ensure-WindowReady + wait_game_window 工具）；
  窗口竞态由 MXU v2.5.3 上层原生解决，无需注入 savedDevice
* version.json 同步依赖指纹；build_release_zip.py 加 version.json 自检
* 根目录瘦身：合并注意事项*.txt/png -> 注意事项.pdf；
  删冗余应用图标.bat（启动器自愈已覆盖）
* 更新弹窗 20 秒无操作自动跳过（防无人值守卡窗）
* README 重写致谢段 + 新建 NOTICE.md（MaaFramework LGPL-3.0 履约）
* resource/pipeline/HuntingArea、Warcraft 适配升级后 MXU
</commit_message>
<xml_diff>
--- a/Verlog.xlsx
+++ b/Verlog.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\BD2MAA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\MABd2v26.09.5\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>更新说明：</t>
   </si>
@@ -169,6 +169,18 @@
   </si>
   <si>
     <t>5.实装新的BAT启动器，可以在启动脚本前自行检查仓库是否存在更新，并可以手动点击更新下载</t>
+  </si>
+  <si>
+    <t>v26.09.5（20260912）</t>
+  </si>
+  <si>
+    <t>1.修正了广场女神像寻路任务点击位置错误的问题</t>
+  </si>
+  <si>
+    <t>v26.09.6（20260913）</t>
+  </si>
+  <si>
+    <t>1.修正了赛季活动自动战斗功能无法进入挑战战斗关的问题</t>
   </si>
 </sst>
 </file>
@@ -791,8 +803,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1109,7 +1124,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="171.125" customWidth="1"/>
@@ -1121,7 +1136,7 @@
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1131,7 +1146,7 @@
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1141,7 +1156,7 @@
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1166,7 +1181,7 @@
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1176,7 +1191,7 @@
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1191,7 +1206,7 @@
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1206,7 +1221,7 @@
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1216,7 +1231,7 @@
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1231,7 +1246,7 @@
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1241,7 +1256,7 @@
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1256,7 +1271,7 @@
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1281,7 +1296,7 @@
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1311,7 +1326,7 @@
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="2" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1338,6 +1353,26 @@
     <row r="60" spans="1:1">
       <c r="A60" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="65" s="1" customFormat="1" spans="1:1">
+      <c r="A65" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: 同步 Verlog.xlsx 至 v26.09.10 定稿
用户在 Excel 中打开 Verlog.xlsx 直接补完的三处（打开期间工作区会出现 `~$Verlog.xlsx`
锁文件，保存后消失）：

- v26.09.9 日期 20260916 -> 20260918（与实际发布日期一致）
- v26.09.10 日期 20260919 -> 20260920
- v26.09.10 新增第 3 条：说明本项目未接入 Mirror酱、软件内 CDK 填写入口已封闭、请勿购买
  CDKEY、更新走 BAT 启动器

打包器不写这个文件（更新内容是人写的），所以这一版发布包里的 Verlog 是上一次保存的快照。
本次提交只带 Verlog.xlsx：与 v26.09.10 发布包逐条比对，206 个条目里只有它一个与磁盘不符。
</commit_message>
<xml_diff>
--- a/Verlog.xlsx
+++ b/Verlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowHeight="11580"/>
+    <workbookView windowWidth="29415" windowHeight="15015"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>更新说明：</t>
   </si>
@@ -192,7 +192,7 @@
     <t>2.更新弹窗 20 秒无操作自动跳过：防无人值守卡在更新窗口</t>
   </si>
   <si>
-    <t>v26.09.9(20260916)</t>
+    <t>v26.09.9(20260918)</t>
   </si>
   <si>
     <t>1.新增商店物品换取，换取物品和时间自选</t>
@@ -210,13 +210,16 @@
     <t>5.优化快速狩猎任务的任务逻辑，防止卡死</t>
   </si>
   <si>
-    <t>v26.09.10(20260919)</t>
+    <t>v26.09.10(20260920)</t>
   </si>
   <si>
     <t>1.修正魔兽快速作战无法识别的问题；</t>
   </si>
   <si>
     <t>2.修正镜中之战PVP因网络卡顿导致的无法进入战斗的问题；</t>
+  </si>
+  <si>
+    <t>3.因本项目目前并没有接入Mirror酱，故封闭了软件内自带的mirror酱填写入口，请勿购买CDKEY，使用BAT启动器即可自动更新</t>
   </si>
 </sst>
 </file>
@@ -1157,7 +1160,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A81"/>
+  <dimension ref="A1:A82"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="171.125" customWidth="1"/>
@@ -1466,6 +1469,11 @@
     <row r="81" spans="1:1">
       <c r="A81" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>